<commit_message>
Stories by god; Chavithi katha = moon + Syamantaka
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tests/M2-stories.xlsx
+++ b/tests/M2-stories.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="2" max="2"/>
@@ -1264,6 +1264,231 @@
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
     </row>
+    <row r="19" ht="72" customHeight="1">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr"/>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mobile</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stories open on a god grid</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stories open on a god grid</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify Stories opens on god cards, not a dropdown</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Open Stories from Home.
+2. Look at the first screen.</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A grid of god cards is shown, using the same card as Puja. Each card shows the god's name and N stories. With one god the grid is still shown.</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="inlineStr"/>
+      <c r="K19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20" ht="72" customHeight="1">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mobile</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Search only above 8 gods</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Search only above 8 gods</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify the search field is hidden until there are more than 8 gods</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Open Stories with the gods that have stories (one god today).
+2. Confirm there is no search field.
+3. In a debug build, Profile, turn on Show story search.
+4. Open Stories again.</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Search is absent with 8 or fewer gods. With the debug flag on, the same search field as Puja appears above the grid.</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="inlineStr"/>
+    </row>
+    <row r="21" ht="72" customHeight="1">
+      <c r="A21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mobile</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">God page order</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">God page order</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify a god's stories follow the order field</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Open Stories, then Ganesha.
+2. Read the story cards from top to bottom.</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Order is the moon story, the Syamantaka jewel, How Ganesha Got His Elephant Head, then the mango story. Each card shows the cover, the title and N min. Read to me is hidden until that language has narration.</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr"/>
+      <c r="K21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22" ht="72" customHeight="1">
+      <c r="A22" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr"/>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mobile</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Back path</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Back path</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify Back walks story, god page, god grid, Home</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Open a story from the Ganesha page.
+2. Press Back.
+3. Press Back again.
+4. Press Back again.
+5. From the grid, press Home.</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Back goes story to the god page, then the god grid, then Home. Home from any of these screens goes to Home.</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr"/>
+      <c r="K22" s="4" t="inlineStr"/>
+    </row>
+    <row r="23" ht="72" customHeight="1">
+      <c r="A23" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr"/>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mobile</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For today on Chavithi</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For today on Chavithi</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify For today on Vinayaka Chavithi is the two-part katha</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Set the debug date to 14 Sep 2026 (Vinayaka Chavithi).
+2. Open Stories.</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Above the god grid, For today shows The Chavithi katha: the moon story, then the Syamantaka jewel. The same card appears on Sankashti.</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr"/>
+      <c r="K23" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Keep the guided step when the katha closes, and record the device checks.
Back from the katha stayed on step 24, and the part title stays readable at 200% font. The walked rows are in the story and puja workbooks.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tests/M2-stories.xlsx
+++ b/tests/M2-stories.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="2" max="2"/>
@@ -454,6 +454,7 @@
     <col width="24.140625" customWidth="1" min="7" max="7"/>
     <col width="26.5703125" customWidth="1" min="8" max="8"/>
     <col width="30.42578125" customWidth="1" min="9" max="9"/>
+    <col width="62" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -512,6 +513,11 @@
           <t>Test Type</t>
         </is>
       </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Result</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="57.95" customHeight="1">
       <c r="A2" s="3" t="n">
@@ -602,6 +608,11 @@
       </c>
       <c r="J3" s="4" t="inlineStr"/>
       <c r="K3" s="4" t="inlineStr"/>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Music starts on. Read to me stays hidden until narration exists, so remembering that switch is waiting for audio.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="57.95" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -646,6 +657,11 @@
       </c>
       <c r="J4" s="4" t="inlineStr"/>
       <c r="K4" s="4" t="inlineStr"/>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">waiting for audio</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="57.95" customHeight="1">
       <c r="A5" s="3" t="n">
@@ -690,6 +706,11 @@
       </c>
       <c r="J5" s="4" t="inlineStr"/>
       <c r="K5" s="4" t="inlineStr"/>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">waiting for audio</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="57.95" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -822,6 +843,11 @@
       </c>
       <c r="J8" s="4" t="inlineStr"/>
       <c r="K8" s="4" t="inlineStr"/>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">waiting for audio</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="57.95" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -866,6 +892,11 @@
       </c>
       <c r="J9" s="4" t="inlineStr"/>
       <c r="K9" s="4" t="inlineStr"/>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">waiting for audio</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="57.95" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -910,6 +941,11 @@
       </c>
       <c r="J10" s="4" t="inlineStr"/>
       <c r="K10" s="4" t="inlineStr"/>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">waiting for audio</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="57.95" customHeight="1">
       <c r="A11" s="3" t="n">
@@ -954,6 +990,11 @@
       </c>
       <c r="J11" s="4" t="inlineStr"/>
       <c r="K11" s="4" t="inlineStr"/>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. The story chip showed the Telugu beat while the chrome stayed English. Switching the app language to Telugu while that story was open changed the chrome and the story (Home became హోమ్, Begin మొదలు). Set back to English.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="57.95" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -998,6 +1039,11 @@
       </c>
       <c r="J12" s="4" t="inlineStr"/>
       <c r="K12" s="4" t="inlineStr"/>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pause stops the music. The voice half is waiting for audio.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="57.95" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -1087,6 +1133,11 @@
       </c>
       <c r="J14" s="4" t="inlineStr"/>
       <c r="K14" s="4" t="inlineStr"/>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. Read to me is hidden in Telugu and in English. Hindi was already hidden.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="57.95" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -1263,6 +1314,11 @@
       </c>
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS for text, pictures and music with airplane mode on. Narration is waiting for audio.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="72" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -1307,6 +1363,11 @@
       </c>
       <c r="J19" s="4" t="inlineStr"/>
       <c r="K19" s="4" t="inlineStr"/>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. Stories opens on god cards. Ganesha shows 4 stories.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="72" customHeight="1">
       <c r="A20" s="3" t="n">
@@ -1353,6 +1414,11 @@
       </c>
       <c r="J20" s="4" t="inlineStr"/>
       <c r="K20" s="4" t="inlineStr"/>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. With one god the field is hidden. Show story search turns it on. zzzz hides the god and For today. gane shows Ganesha.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="72" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -1397,6 +1463,11 @@
       </c>
       <c r="J21" s="4" t="inlineStr"/>
       <c r="K21" s="4" t="inlineStr"/>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. The god page leads with Ganesha and the Moon, then The Syamantaka Jewel, which is the order in the story files.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="72" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -1444,6 +1515,11 @@
       </c>
       <c r="J22" s="4" t="inlineStr"/>
       <c r="K22" s="4" t="inlineStr"/>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. Back from the god page returns to the grid. Back from a story returns to the screen it was opened from.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="72" customHeight="1">
       <c r="A23" s="3" t="n">
@@ -1488,6 +1564,109 @@
       </c>
       <c r="J23" s="4" t="inlineStr"/>
       <c r="K23" s="4" t="inlineStr"/>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS on Vinayaka Chavithi. For today is The Chavithi katha: the moon, then the Syamantaka jewel, with Continue · part 2 of 2. Sankashti was not opened this pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="72" customHeight="1">
+      <c r="A24" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mobile</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">200% font on the god grid, god page and katha card</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">200% font on the god grid, god page and katha card</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify the god grid, the god page and the katha card at 200% font</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Set the system font scale to 2.0.
+2. Open Stories, the Ganesha page, and the Chavithi katha.</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text stays readable and the screens scroll. Nothing is clipped to a single letter.</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr"/>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. At font scale 2.0 the grid, the god page and the katha card stay readable and scroll. The part title had collapsed to one letter per line in the top row; it now sits on its own line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="72" customHeight="1">
+      <c r="A25" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mobile</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TalkBack on the god grid, god page and katha card</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TalkBack on the god grid, god page and katha card</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify TalkBack names for the god card and the katha card</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Turn TalkBack on.
+2. Open Stories and focus the Ganesha card and the Chavithi katha card.</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The god card is announced as the god and the story count. The katha card is announced as Chavithi katha, 2 parts.</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr"/>
+      <c r="K25" s="4" t="inlineStr"/>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS for the names. With TalkBack on, the tree reads Ganesha, 4 stories and Chavithi katha, 2 parts. A system notification sheet blocked the spoken double-tap and was closed without allowing notifications.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Record the story checks that do not need narration.
The moon story turns by hand, pauses on lock, and ends with the puja and more stories. The voice rows stay waiting for audio.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tests/M2-stories.xlsx
+++ b/tests/M2-stories.xlsx
@@ -563,6 +563,11 @@
       </c>
       <c r="J2" s="4" t="inlineStr"/>
       <c r="K2" s="4" t="inlineStr"/>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. No age choice. The moon story's first beat and its last line are each one sentence.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="57.95" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -755,6 +760,11 @@
       </c>
       <c r="J6" s="4" t="inlineStr"/>
       <c r="K6" s="4" t="inlineStr"/>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. Swiping moved to the next beat at once. No voice was playing.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="57.95" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -799,6 +809,11 @@
       </c>
       <c r="J7" s="4" t="inlineStr"/>
       <c r="K7" s="4" t="inlineStr"/>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. Read to me is hidden, so the page stays until it is turned. Music plays.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="57.95" customHeight="1">
       <c r="A8" s="3" t="n">
@@ -1041,7 +1056,7 @@
       <c r="K12" s="4" t="inlineStr"/>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pause stops the music. The voice half is waiting for audio.</t>
+          <t xml:space="preserve">PASS for the music. Pause, and locking the screen, both leave the control on Play and the bed does not start again. The voice is waiting for audio.</t>
         </is>
       </c>
     </row>
@@ -1088,6 +1103,11 @@
       </c>
       <c r="J13" s="4" t="inlineStr"/>
       <c r="K13" s="4" t="inlineStr"/>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. Sleeping the screen changed Pause to Play. Waking the screen did not start the music.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="57.95" customHeight="1">
       <c r="A14" s="3" t="n">
@@ -1182,6 +1202,11 @@
       </c>
       <c r="J15" s="4" t="inlineStr"/>
       <c r="K15" s="4" t="inlineStr"/>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pictures are supplied for these beats, so the symbol was not what showed. A missing picture still uses the deity symbol.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="57.95" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -1226,6 +1251,11 @@
       </c>
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. The last beat offers Do the puja and More stories of Ganesha. No score.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="57.95" customHeight="1">
       <c r="A17" s="3" t="n">

</xml_diff>